<commit_message>
Added two additional records, waiting on other travel to do today and will add the Touch In and Touch Out times in due course.
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCA477E6-B106-425B-97B4-C16811D903A8}"/>
+  <xr:revisionPtr revIDLastSave="102" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF84AF8E-82F4-447C-A8B2-E63E42C12F55}"/>
   <bookViews>
-    <workbookView xWindow="10260" yWindow="990" windowWidth="21600" windowHeight="11835" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -598,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1170,6 +1170,43 @@
         <v>14</v>
       </c>
     </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46302</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3">
+        <v>46302</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added more records to the spreadsheet for 07/10/2026 and begun adding records for 08/10/2026.
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="102" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF84AF8E-82F4-447C-A8B2-E63E42C12F55}"/>
+  <xr:revisionPtr revIDLastSave="152" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{865ADC92-E15E-4329-905F-803C19B26CA8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -598,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -993,7 +993,7 @@
       <c r="B15" s="3">
         <v>46300</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="7">
         <v>24</v>
       </c>
       <c r="D15" s="4">
@@ -1180,6 +1180,9 @@
       <c r="C23" s="10" t="s">
         <v>8</v>
       </c>
+      <c r="D23" s="4">
+        <v>0.5444444444444444</v>
+      </c>
       <c r="E23" t="s">
         <v>11</v>
       </c>
@@ -1200,10 +1203,142 @@
       <c r="C24" s="9" t="s">
         <v>10</v>
       </c>
+      <c r="D24" s="4">
+        <v>0.55902777777777779</v>
+      </c>
       <c r="E24" t="s">
         <v>11</v>
       </c>
+      <c r="F24" s="4">
+        <v>0.58958333333333335</v>
+      </c>
       <c r="G24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3">
+        <v>46302</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0.7583333333333333</v>
+      </c>
+      <c r="E25" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0.76666666666666672</v>
+      </c>
+      <c r="G25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3">
+        <v>46302</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="4">
+        <v>0.78263888888888888</v>
+      </c>
+      <c r="E26" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0.81388888888888888</v>
+      </c>
+      <c r="G26" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3">
+        <v>46302</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="4">
+        <v>0.81805555555555554</v>
+      </c>
+      <c r="E27" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3">
+        <v>46303</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3">
+        <v>46303</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s">
+        <v>11</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3">
+        <v>46303</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Entered all the data values for 08/10/2026 and begun to enter values for 09/10/2026.
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="152" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{865ADC92-E15E-4329-905F-803C19B26CA8}"/>
+  <xr:revisionPtr revIDLastSave="177" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50895534-9C3C-4F41-8913-55FDAA981B63}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="31">
   <si>
     <t>ID</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t xml:space="preserve">  as you only touch in on these services.</t>
+  </si>
+  <si>
+    <t>LU</t>
   </si>
 </sst>
 </file>
@@ -151,7 +154,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -224,6 +227,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFAE1E1E"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -237,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -253,6 +262,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -261,9 +271,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFAE1E1E"/>
+      <color rgb="FF0F00CC"/>
       <color rgb="FFFF3300"/>
-      <color rgb="FF0F00CC"/>
-      <color rgb="FFAE1E1E"/>
     </mruColors>
   </colors>
   <extLst>
@@ -598,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1295,6 +1305,9 @@
       <c r="C28" s="10" t="s">
         <v>8</v>
       </c>
+      <c r="D28" s="4">
+        <v>0.53888888888888886</v>
+      </c>
       <c r="E28" t="s">
         <v>11</v>
       </c>
@@ -1315,8 +1328,14 @@
       <c r="C29" s="9" t="s">
         <v>10</v>
       </c>
+      <c r="D29" s="4">
+        <v>0.55277777777777781</v>
+      </c>
       <c r="E29" t="s">
         <v>11</v>
+      </c>
+      <c r="F29" s="4">
+        <v>0.58263888888888893</v>
       </c>
       <c r="G29" t="s">
         <v>15</v>
@@ -1332,6 +1351,9 @@
       <c r="C30" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="D30" s="4">
+        <v>0.58750000000000002</v>
+      </c>
       <c r="E30" t="s">
         <v>11</v>
       </c>
@@ -1339,6 +1361,66 @@
         <v>13</v>
       </c>
       <c r="G30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3">
+        <v>46303</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D31" s="4">
+        <v>0.75694444444444442</v>
+      </c>
+      <c r="E31" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="4">
+        <v>0.76388888888888884</v>
+      </c>
+      <c r="G31" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3">
+        <v>46304</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="E32" t="s">
+        <v>11</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3">
+        <v>46304</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added all relevant data for 09/10/2026, no transport was taken on 10/10/2026 so not added to the spreadsheet.
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="177" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50895534-9C3C-4F41-8913-55FDAA981B63}"/>
+  <xr:revisionPtr revIDLastSave="213" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76CE8172-121F-42A8-89FE-52F8BCF908AE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="31">
   <si>
     <t>ID</t>
   </si>
@@ -608,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R33"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1397,8 +1397,14 @@
       <c r="C32" s="11" t="s">
         <v>30</v>
       </c>
+      <c r="D32" s="4">
+        <v>0.41805555555555557</v>
+      </c>
       <c r="E32" t="s">
         <v>11</v>
+      </c>
+      <c r="F32" s="4">
+        <v>0.42499999999999999</v>
       </c>
       <c r="G32" t="s">
         <v>15</v>
@@ -1414,6 +1420,9 @@
       <c r="C33" s="15" t="s">
         <v>7</v>
       </c>
+      <c r="D33" s="4">
+        <v>0.4284722222222222</v>
+      </c>
       <c r="E33" t="s">
         <v>11</v>
       </c>
@@ -1422,6 +1431,98 @@
       </c>
       <c r="G33" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3">
+        <v>46304</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="4">
+        <v>0.67152777777777772</v>
+      </c>
+      <c r="E34" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3">
+        <v>46304</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="4">
+        <v>0.67777777777777781</v>
+      </c>
+      <c r="E35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="4">
+        <v>0.70347222222222228</v>
+      </c>
+      <c r="G35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46304</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="4">
+        <v>0.70902777777777781</v>
+      </c>
+      <c r="E36" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3">
+        <v>46304</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="4">
+        <v>0.74722222222222223</v>
+      </c>
+      <c r="E37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added the data for 11/10/2026, no journeys were made on 09 or 10 and will begin adding data for 12/10/2026 shortly
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="213" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76CE8172-121F-42A8-89FE-52F8BCF908AE}"/>
+  <xr:revisionPtr revIDLastSave="260" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27BAAD79-D8E1-4FF8-A6AD-C7F7A8FB4F80}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="31">
   <si>
     <t>ID</t>
   </si>
@@ -138,7 +138,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -149,6 +149,12 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -246,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -263,6 +269,7 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -272,8 +279,8 @@
   <colors>
     <mruColors>
       <color rgb="FFAE1E1E"/>
+      <color rgb="FFFF3300"/>
       <color rgb="FF0F00CC"/>
-      <color rgb="FFFF3300"/>
     </mruColors>
   </colors>
   <extLst>
@@ -608,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R37"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1525,6 +1532,121 @@
         <v>14</v>
       </c>
     </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3">
+        <v>46306</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="4">
+        <v>0.31944444444444442</v>
+      </c>
+      <c r="E38" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3">
+        <v>46306</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="4">
+        <v>0.33263888888888887</v>
+      </c>
+      <c r="E39" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="4">
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3">
+        <v>46306</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="4">
+        <v>0.36249999999999999</v>
+      </c>
+      <c r="E40" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3">
+        <v>46306</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="4">
+        <v>0.67152777777777772</v>
+      </c>
+      <c r="E41" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="G41" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3">
+        <v>46306</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="4">
+        <v>0.70208333333333328</v>
+      </c>
+      <c r="E42" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Changed the 11/10 journeys to 12/10 as no journeys were done on 11/10 and added the journeys for 13/10 as well.
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="260" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27BAAD79-D8E1-4FF8-A6AD-C7F7A8FB4F80}"/>
+  <xr:revisionPtr revIDLastSave="318" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B02B77C0-7D74-419C-B727-CE2184CEEB9D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="31">
   <si>
     <t>ID</t>
   </si>
@@ -138,7 +138,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,8 +159,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -239,6 +247,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -249,10 +263,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -270,16 +285,18 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="20" fontId="2" fillId="14" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF3300"/>
       <color rgb="FFAE1E1E"/>
-      <color rgb="FFFF3300"/>
       <color rgb="FF0F00CC"/>
     </mruColors>
   </colors>
@@ -292,10 +309,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -615,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1537,7 +1550,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="C38" s="10" t="s">
         <v>8</v>
@@ -1560,7 +1573,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>10</v>
@@ -1583,7 +1596,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="C40" s="15" t="s">
         <v>7</v>
@@ -1606,7 +1619,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>10</v>
@@ -1629,7 +1642,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>7</v>
@@ -1644,6 +1657,121 @@
         <v>13</v>
       </c>
       <c r="G42" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" s="4">
+        <v>0.31736111111111109</v>
+      </c>
+      <c r="E43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G43" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="4">
+        <v>0.33402777777777776</v>
+      </c>
+      <c r="E44" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="4">
+        <v>0.36041666666666666</v>
+      </c>
+      <c r="G44" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" s="4">
+        <v>0.3659722222222222</v>
+      </c>
+      <c r="E45" t="s">
+        <v>12</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G45" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D46" s="17">
+        <v>0.71388888888888891</v>
+      </c>
+      <c r="E46" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="4">
+        <v>0.74236111111111114</v>
+      </c>
+      <c r="G46" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3">
+        <v>46308</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" s="4">
+        <v>0.74722222222222223</v>
+      </c>
+      <c r="E47" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G47" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added all records for 14/10/2026 and begun adding records for 15/10/2026
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="318" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B02B77C0-7D74-419C-B727-CE2184CEEB9D}"/>
+  <xr:revisionPtr revIDLastSave="364" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16341FB4-255F-46F9-A4E8-00B7C7745936}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="31">
   <si>
     <t>ID</t>
   </si>
@@ -309,6 +309,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -628,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R47"/>
+  <dimension ref="A1:R53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1775,6 +1779,132 @@
         <v>14</v>
       </c>
     </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3">
+        <v>46309</v>
+      </c>
+      <c r="C48" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" s="4">
+        <v>0.56388888888888888</v>
+      </c>
+      <c r="E48" t="s">
+        <v>11</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G48" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3">
+        <v>46309</v>
+      </c>
+      <c r="C49" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49" s="4">
+        <v>0.7368055555555556</v>
+      </c>
+      <c r="E49" t="s">
+        <v>11</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3">
+        <v>46309</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" s="4">
+        <v>0.75972222222222219</v>
+      </c>
+      <c r="E50" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G50" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3">
+        <v>46310</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3">
+        <v>46310</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3">
+        <v>46310</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E53" t="s">
+        <v>11</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added the full records for 15/10 and will begin adding 16/10.
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="364" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16341FB4-255F-46F9-A4E8-00B7C7745936}"/>
+  <xr:revisionPtr revIDLastSave="394" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6CF41C6-D1C0-44D2-9723-3F6910728DEF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="32">
   <si>
     <t>ID</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t>LU</t>
+  </si>
+  <si>
+    <t>NR</t>
   </si>
 </sst>
 </file>
@@ -632,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R53"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1858,6 +1861,9 @@
       <c r="C51" s="10" t="s">
         <v>8</v>
       </c>
+      <c r="D51" s="4">
+        <v>0.51597222222222228</v>
+      </c>
       <c r="E51" t="s">
         <v>11</v>
       </c>
@@ -1878,8 +1884,14 @@
       <c r="C52" s="9" t="s">
         <v>10</v>
       </c>
+      <c r="D52" s="4">
+        <v>0.52986111111111112</v>
+      </c>
       <c r="E52" t="s">
         <v>11</v>
+      </c>
+      <c r="F52" s="4">
+        <v>0.55694444444444446</v>
       </c>
       <c r="G52" t="s">
         <v>15</v>
@@ -1895,6 +1907,9 @@
       <c r="C53" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="D53" s="4">
+        <v>0.55902777777777779</v>
+      </c>
       <c r="E53" t="s">
         <v>11</v>
       </c>
@@ -1903,6 +1918,75 @@
       </c>
       <c r="G53" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3">
+        <v>46310</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D54" s="4">
+        <v>0.7583333333333333</v>
+      </c>
+      <c r="E54" t="s">
+        <v>11</v>
+      </c>
+      <c r="F54" s="4">
+        <v>0.76666666666666672</v>
+      </c>
+      <c r="G54" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3">
+        <v>46310</v>
+      </c>
+      <c r="C55" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D55" s="4">
+        <v>0.83611111111111114</v>
+      </c>
+      <c r="E55" t="s">
+        <v>11</v>
+      </c>
+      <c r="F55" s="4">
+        <v>0.85347222222222219</v>
+      </c>
+      <c r="G55" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3">
+        <v>46310</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" s="4">
+        <v>0.85555555555555551</v>
+      </c>
+      <c r="E56" t="s">
+        <v>11</v>
+      </c>
+      <c r="F56" t="s">
+        <v>13</v>
+      </c>
+      <c r="G56" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added all journeys for 16/10/2026 and will begin working on my Processing sketch by tommorow evening.
</commit_message>
<xml_diff>
--- a/Dear Data Spreadsheet.xlsx
+++ b/Dear Data Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/peter_nurden_city_ac_uk/Documents/MSci Computer Science (G401)/Year 1/Programming in Java - IN1007/Creative Coding/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="394" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6CF41C6-D1C0-44D2-9723-3F6910728DEF}"/>
+  <xr:revisionPtr revIDLastSave="434" documentId="8_{E8A74F6E-D15F-44DE-819A-224ADEADB942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBE43505-7AFF-4010-A7FF-D5CDFEA69149}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72960D65-58F2-4B8C-AE2A-CBBD65864024}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="32">
   <si>
     <t>ID</t>
   </si>
@@ -635,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF54C2F-01A9-4473-A27C-C7817089220B}">
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:R61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1989,6 +1989,121 @@
         <v>14</v>
       </c>
     </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3">
+        <v>46311</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" s="4">
+        <v>0.37152777777777779</v>
+      </c>
+      <c r="E57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G57" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3">
+        <v>46311</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D58" s="4">
+        <v>0.38750000000000001</v>
+      </c>
+      <c r="E58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" s="4">
+        <v>0.41458333333333336</v>
+      </c>
+      <c r="G58" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3">
+        <v>46311</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F59" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3">
+        <v>46311</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D60" s="4">
+        <v>0.67500000000000004</v>
+      </c>
+      <c r="E60" t="s">
+        <v>11</v>
+      </c>
+      <c r="F60" s="4">
+        <v>0.70347222222222228</v>
+      </c>
+      <c r="G60" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3">
+        <v>46311</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" s="4">
+        <v>0.7055555555555556</v>
+      </c>
+      <c r="E61" t="s">
+        <v>11</v>
+      </c>
+      <c r="F61" t="s">
+        <v>13</v>
+      </c>
+      <c r="G61" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>